<commit_message>
Correct 솔브레인홀딩스·한화머시너리 classification against disclosure data
- 한화머시너리앤서비스홀딩스: 산업기계가 아니라 2026-08-01 (주)한화
  인적분할 신설 지주. 한화비전 → 한화세미텍(HBM TC본더) 2단 룩스루가
  주력이므로 팀 2 → 팀 1, 테마 반도체·AI
- (주)한화: 같은 분할로 모멘텀·비전이 이탈, 자체 사업은 화약·유도무기와
  건설만 남음 → 테마 방산·건설
- 솔브레인홀딩스: 순수지주(2020 인적분할 투자사업부문). 솔브레인 44.9%,
  바이오헬스케어 연결 매출 11%
- 팀 비중 17.32 / 16.87 / 15.36%

DART 접근이 차단되어 KRX·증권정보 2차 자료로 확인. 솔브레인홀딩스
바이오헬스케어의 직접 영위 여부는 사업보고서 원문 확인이 필요하다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jphTyMQLHbxpFNoQ68jkL
</commit_message>
<xml_diff>
--- a/docs/26-2/data/ICOK_담당산업_스크리닝_20260915.xlsx
+++ b/docs/26-2/data/ICOK_담당산업_스크리닝_20260915.xlsx
@@ -1281,7 +1281,7 @@
         <v>0.01056536581304022</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.0734229604263872</v>
+        <v>0.07347179509010925</v>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
@@ -1320,7 +1320,7 @@
         <v>0.002678260663048011</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.02710513322945303</v>
+        <v>0.02712316124219883</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -1359,7 +1359,7 @@
         <v>0.001869436878772927</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.01074895213158637</v>
+        <v>0.01075610141376815</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
         <v>0.001578987355546556</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.09172580214650965</v>
+        <v>0.09178681029268691</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -1437,7 +1437,7 @@
         <v>0.001475877119536982</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.004047784533016677</v>
+        <v>0.004050476772546945</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -1476,7 +1476,7 @@
         <v>0.001199452315751969</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.02845933192319619</v>
+        <v>0.02847826063290978</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
         <v>0.001079846131773961</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.01269561275384217</v>
+        <v>0.01270405678791514</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -1554,7 +1554,7 @@
         <v>0.0008936097161851883</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.06866210564369638</v>
+        <v>0.06870777379464106</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -1593,7 +1593,7 @@
         <v>0.0008458332571776441</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.01470575143986718</v>
+        <v>0.01471553244600171</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -1632,7 +1632,7 @@
         <v>0.0007582779421362232</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.09944896657176364</v>
+        <v>0.09951511150533529</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
         <v>0.0006494832421480894</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>0.01891646300322483</v>
+        <v>0.01892904461399356</v>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
@@ -1710,7 +1710,7 @@
         <v>0.0006073829859084085</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>0.007998236034920565</v>
+        <v>0.008003555776386541</v>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
@@ -1749,7 +1749,7 @@
         <v>0.000536538034803962</v>
       </c>
       <c r="G22" s="17" t="n">
-        <v>0.01546748820509771</v>
+        <v>0.01547777585327662</v>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
         <v>0.000448549193955747</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>0.004538681559498574</v>
+        <v>0.004541700301679664</v>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         <v>0.0004280495628759759</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>0.02175181651824958</v>
+        <v>0.02176628396329461</v>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
@@ -1866,7 +1866,7 @@
         <v>0.0003137361863875837</v>
       </c>
       <c r="G25" s="17" t="n">
-        <v>0.01115097986879137</v>
+        <v>0.01115839654538547</v>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         <v>0.0001537341841404777</v>
       </c>
       <c r="G26" s="17" t="n">
-        <v>0.01470575143986718</v>
+        <v>0.01471553244600171</v>
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
         <v>0.0001378292882464421</v>
       </c>
       <c r="G27" s="17" t="n">
-        <v>0.001299184371809848</v>
+        <v>0.001300048477963316</v>
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
@@ -1983,7 +1983,7 @@
         <v>0.0001375776968297665</v>
       </c>
       <c r="G28" s="26" t="n">
-        <v>0.001436720176643139</v>
+        <v>0.001437675759832397</v>
       </c>
       <c r="H28" s="22" t="inlineStr">
         <is>
@@ -2492,7 +2492,7 @@
         <v>0.01029119575651107</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.2249239392889037</v>
+        <v>0.2250735394258966</v>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
@@ -2531,7 +2531,7 @@
         <v>0.002771636188780124</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.1419792692971349</v>
+        <v>0.142073701744851</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -2570,7 +2570,7 @@
         <v>0.002487727291368166</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.02568745647194065</v>
+        <v>0.02570454156754831</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -2609,7 +2609,7 @@
         <v>0.002472295162031734</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.01474807014904665</v>
+        <v>0.01475787930196142</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -2648,7 +2648,7 @@
         <v>0.002360882972536231</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.02729556742076066</v>
+        <v>0.02731372209401756</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -2687,7 +2687,7 @@
         <v>0.0004004148743212</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.01610226884278981</v>
+        <v>0.01611297869267237</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -2726,7 +2726,7 @@
         <v>0.0001745045576253579</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.004898390587524102</v>
+        <v>0.004901648577337259</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -2765,7 +2765,7 @@
         <v>0.0001484543317312726</v>
       </c>
       <c r="G17" s="26" t="n">
-        <v>0.01527705401379007</v>
+        <v>0.01528721500145789</v>
       </c>
       <c r="H17" s="22" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
         <v>0.004939488087684244</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.07024905723792665</v>
+        <v>0.07029578089313046</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -3320,7 +3320,7 @@
         <v>0.004497624653994468</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.02998280545365725</v>
+        <v>0.0300027474474596</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -3359,7 +3359,7 @@
         <v>0.004459821917110226</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.2407934552312064</v>
+        <v>0.2409536104107906</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
         <v>0.003657062236996178</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.004369406722780679</v>
+        <v>0.004372312877840795</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -3437,7 +3437,7 @@
         <v>0.003598474669508337</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.0574476477111358</v>
+        <v>0.05748585696531602</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -3476,7 +3476,7 @@
         <v>0.003143214368390162</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.03146396027493883</v>
+        <v>0.0314848874060497</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -3515,7 +3515,7 @@
         <v>0.0020291176325768</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.006210270572087792</v>
+        <v>0.006214401112088491</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -3554,7 +3554,7 @@
         <v>0.001813365976470995</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.01161648566976558</v>
+        <v>0.01162421196094236</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -3593,7 +3593,7 @@
         <v>0.001205513791345966</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.006040995735369897</v>
+        <v>0.006045013688249622</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -3632,7 +3632,7 @@
         <v>0.0008806861785787587</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>0.007437513138292535</v>
+        <v>0.007442459934920288</v>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
@@ -3671,7 +3671,7 @@
         <v>0.000812965279401227</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>0.01847211655684035</v>
+        <v>0.01848440262641653</v>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
@@ -3710,7 +3710,7 @@
         <v>0.00071335404163133</v>
       </c>
       <c r="G22" s="17" t="n">
-        <v>0.04305928659011468</v>
+        <v>0.04308792593901219</v>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
@@ -3749,7 +3749,7 @@
         <v>0.000579089841310139</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>0.02594136872701749</v>
+        <v>0.02595862270330661</v>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
@@ -3788,7 +3788,7 @@
         <v>0.0005700901910299061</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>0.001201851340697058</v>
+        <v>0.001202650709255967</v>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
@@ -3827,7 +3827,7 @@
         <v>0.000517215062984121</v>
       </c>
       <c r="G25" s="17" t="n">
-        <v>0.01362662435579059</v>
+        <v>0.01363568761902892</v>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
@@ -3866,7 +3866,7 @@
         <v>0.0004176828699802094</v>
       </c>
       <c r="G26" s="17" t="n">
-        <v>0.05078245101536866</v>
+        <v>0.05081622715166057</v>
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
@@ -3905,7 +3905,7 @@
         <v>0.0003687930250764813</v>
       </c>
       <c r="G27" s="17" t="n">
-        <v>0.01375358048332901</v>
+        <v>0.01376272818690807</v>
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
@@ -3944,7 +3944,7 @@
         <v>0.0003071001811405816</v>
       </c>
       <c r="G28" s="17" t="n">
-        <v>0.01517125724084139</v>
+        <v>0.0151813478615586</v>
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v>0.000303742374501905</v>
       </c>
       <c r="G29" s="17" t="n">
-        <v>0.00775490345713859</v>
+        <v>0.007760061354618167</v>
       </c>
       <c r="H29" s="13" t="inlineStr">
         <is>
@@ -4022,7 +4022,7 @@
         <v>0.0003019288509991665</v>
       </c>
       <c r="G30" s="17" t="n">
-        <v>0.01136257341468874</v>
+        <v>0.01137013082518405</v>
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
@@ -4061,7 +4061,7 @@
         <v>0.0002912146239897681</v>
       </c>
       <c r="G31" s="17" t="n">
-        <v>0.009151420860061227</v>
+        <v>0.009157507601288832</v>
       </c>
       <c r="H31" s="13" t="inlineStr">
         <is>
@@ -4100,7 +4100,7 @@
         <v>0.0002640765468507437</v>
       </c>
       <c r="G32" s="17" t="n">
-        <v>0.06876790241664507</v>
+        <v>0.06881364093454036</v>
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
@@ -4139,7 +4139,7 @@
         <v>0.0002199209389406541</v>
       </c>
       <c r="G33" s="17" t="n">
-        <v>0.009606346983740572</v>
+        <v>0.009612736302855791</v>
       </c>
       <c r="H33" s="13" t="inlineStr">
         <is>
@@ -4178,7 +4178,7 @@
         <v>0.0001896049242503972</v>
       </c>
       <c r="G34" s="17" t="n">
-        <v>0.1919153461289141</v>
+        <v>0.1920429917773173</v>
       </c>
       <c r="H34" s="13" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         <v>0.0001760375754739821</v>
       </c>
       <c r="G35" s="17" t="n">
-        <v>0.01146837018763742</v>
+        <v>0.01147599796508335</v>
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
@@ -4256,7 +4256,7 @@
         <v>0.0001745629493646012</v>
       </c>
       <c r="G36" s="17" t="n">
-        <v>0.01068547406781716</v>
+        <v>0.01069258112982858</v>
       </c>
       <c r="H36" s="13" t="inlineStr">
         <is>
@@ -4295,7 +4295,7 @@
         <v>0.0001413100742716281</v>
       </c>
       <c r="G37" s="26" t="n">
-        <v>0.03554771571075806</v>
+        <v>0.0355713590061624</v>
       </c>
       <c r="H37" s="22" t="inlineStr">
         <is>
@@ -4561,7 +4561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>2.24%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="C5" s="9" t="n"/>
@@ -4662,7 +4662,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>626,571원</t>
+          <t>623,430원</t>
         </is>
       </c>
       <c r="F5" s="9" t="n"/>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I5" s="9" t="n"/>
@@ -4692,7 +4692,7 @@
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>순수지주를 재료 기준으로 묶었다. 두산은 자체 사업(전자BG 하이엔드 CCL)과 자회사(두산에너빌리티 가스터빈·SMR)가 모두 AI 데이터센터로 모인다 — 팀 1의 이수페타시스·대덕전자와 재료가 겹치므로 합산 노출을 확인한다. 하림지주는 육계가 아니라 팬오션(벌크 해운)이 NAV의 대부분이라 이 팀으로 옮겼다.</t>
+          <t>순수지주를 재료 기준으로 묶었다. 두산은 자체 사업(전자BG 하이엔드 CCL)과 자회사(두산에너빌리티 가스터빈·SMR)가 모두 AI 데이터센터로 모인다 — 팀 1의 이수페타시스·대덕전자와 재료가 겹치므로 합산 노출을 확인한다. 하림지주는 육계가 아니라 팬오션(벌크 해운)이 NAV의 대부분이라 이 팀으로 옮겼다. (주)한화는 인적분할로 모멘텀·비전이 빠져나가 자체 사업이 화약·유도무기와 건설만 남았다.</t>
         </is>
       </c>
     </row>
@@ -4816,7 +4816,7 @@
         <v>0.007487001385355655</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.1163764502435532</v>
+        <v>0.1164538538892222</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -4867,7 +4867,7 @@
         <v>0.003919165856528693</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.2727440806617092</v>
+        <v>0.272925486660377</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -4918,7 +4918,7 @@
         <v>0.003337049220272115</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.04760854782690812</v>
+        <v>0.04764021295468179</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -4969,7 +4969,7 @@
         <v>0.002007525080872798</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.02435441713278722</v>
+        <v>0.02437061560481722</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>0.001777887643869175</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.06421864117985163</v>
+        <v>0.06426135391887076</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -5071,7 +5071,7 @@
         <v>0.00173107474243654</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.02922106868842672</v>
+        <v>0.02924050404018469</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -5099,7 +5099,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>방산·기계</t>
+          <t>방산·건설</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -5122,7 +5122,7 @@
         <v>0.001372748859067707</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.02900947514252935</v>
+        <v>0.0290287697603861</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -5135,12 +5135,12 @@
       <c r="L17" s="5" t="n"/>
       <c r="M17" s="36" t="inlineStr">
         <is>
-          <t>글로벌부문 — 화약 · 유도무기 / 모멘텀 — 2차전지·태양광 장비</t>
+          <t>글로벌부문 — 화약 · 유도무기 / 건설부문</t>
         </is>
       </c>
       <c r="N17" s="36" t="inlineStr">
         <is>
-          <t>한화에어로스페이스 · 한화솔루션</t>
+          <t>한화에어로스페이스 · 한화오션 · 한화솔루션 · 한화생명</t>
         </is>
       </c>
       <c r="O17" s="5" t="n"/>
@@ -5173,7 +5173,7 @@
         <v>0.0002363725767789877</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.002378311455886432</v>
+        <v>0.002379893304936103</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -5224,7 +5224,7 @@
         <v>0.0002104994036505181</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.01132025470550926</v>
+        <v>0.01132778396922434</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -5250,142 +5250,114 @@
       <c r="Q19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>화학</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>SK디스커버리</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="22" t="inlineStr">
         <is>
           <t>006120</t>
         </is>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="D20" s="23" t="n">
         <v>56900</v>
       </c>
-      <c r="E20" s="15" t="n">
+      <c r="E20" s="24" t="n">
         <v>0.990842</v>
       </c>
-      <c r="F20" s="16" t="n">
+      <c r="F20" s="25" t="n">
         <v>0.0001860353302102206</v>
       </c>
-      <c r="G20" s="17" t="n">
-        <v>0.01203967276156032</v>
-      </c>
-      <c r="H20" s="13" t="inlineStr">
-        <is>
-          <t>가능</t>
-        </is>
-      </c>
-      <c r="I20" s="19" t="n"/>
-      <c r="J20" s="19" t="n"/>
-      <c r="K20" s="19" t="n"/>
-      <c r="L20" s="19" t="n"/>
-      <c r="M20" s="36" t="inlineStr">
+      <c r="G20" s="26" t="n">
+        <v>0.01204768052053953</v>
+      </c>
+      <c r="H20" s="22" t="inlineStr">
+        <is>
+          <t>가능</t>
+        </is>
+      </c>
+      <c r="I20" s="34" t="n"/>
+      <c r="J20" s="34" t="n"/>
+      <c r="K20" s="34" t="n"/>
+      <c r="L20" s="34" t="n"/>
+      <c r="M20" s="37" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N20" s="36" t="inlineStr">
+      <c r="N20" s="37" t="inlineStr">
         <is>
           <t>SK케미칼 · SK가스 · SK바이오사이언스</t>
         </is>
       </c>
-      <c r="O20" s="19" t="n"/>
-      <c r="P20" s="19" t="n"/>
-      <c r="Q20" s="19" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="21" t="inlineStr">
-        <is>
-          <t>방산·기계</t>
-        </is>
-      </c>
-      <c r="B21" s="21" t="inlineStr">
-        <is>
-          <t>한화머시너리앤서비스홀딩스</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="inlineStr">
-        <is>
-          <t>0220W0</t>
-        </is>
-      </c>
-      <c r="D21" s="23" t="n">
-        <v>7070</v>
-      </c>
-      <c r="E21" s="24" t="n">
-        <v>0.597525</v>
-      </c>
-      <c r="F21" s="25" t="n">
-        <v>0.0001121881800366376</v>
-      </c>
-      <c r="G21" s="26" t="n">
-        <v>0.001495966369494402</v>
-      </c>
-      <c r="H21" s="22" t="inlineStr">
-        <is>
-          <t>가능</t>
-        </is>
-      </c>
-      <c r="I21" s="27" t="n"/>
-      <c r="J21" s="27" t="n"/>
-      <c r="K21" s="27" t="n"/>
-      <c r="L21" s="27" t="n"/>
-      <c r="M21" s="37" t="inlineStr">
-        <is>
-          <t>산업기계 · 유지보수 서비스</t>
-        </is>
-      </c>
-      <c r="N21" s="37" t="inlineStr">
-        <is>
-          <t>기계 계열</t>
-        </is>
-      </c>
-      <c r="O21" s="27" t="n"/>
-      <c r="P21" s="27" t="n"/>
-      <c r="Q21" s="27" t="n"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="O20" s="34" t="n"/>
+      <c r="P20" s="34" t="n"/>
+      <c r="Q20" s="34" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="28" t="inlineStr">
         <is>
           <t>선정 결과</t>
         </is>
       </c>
-      <c r="B23" s="28" t="n"/>
-      <c r="C23" s="28" t="n"/>
-      <c r="D23" s="28" t="n"/>
-      <c r="E23" s="28" t="n"/>
-      <c r="F23" s="28" t="n"/>
-      <c r="G23" s="28" t="n"/>
-      <c r="H23" s="28" t="n"/>
-      <c r="I23" s="28" t="n"/>
-      <c r="J23" s="28" t="n"/>
-      <c r="K23" s="28" t="n"/>
-      <c r="L23" s="28" t="n"/>
-      <c r="M23" s="28" t="n"/>
-      <c r="N23" s="28" t="n"/>
-      <c r="O23" s="28" t="n"/>
-      <c r="P23" s="28" t="n"/>
-      <c r="Q23" s="28" t="n"/>
+      <c r="B22" s="28" t="n"/>
+      <c r="C22" s="28" t="n"/>
+      <c r="D22" s="28" t="n"/>
+      <c r="E22" s="28" t="n"/>
+      <c r="F22" s="28" t="n"/>
+      <c r="G22" s="28" t="n"/>
+      <c r="H22" s="28" t="n"/>
+      <c r="I22" s="28" t="n"/>
+      <c r="J22" s="28" t="n"/>
+      <c r="K22" s="28" t="n"/>
+      <c r="L22" s="28" t="n"/>
+      <c r="M22" s="28" t="n"/>
+      <c r="N22" s="28" t="n"/>
+      <c r="O22" s="28" t="n"/>
+      <c r="P22" s="28" t="n"/>
+      <c r="Q22" s="28" t="n"/>
+    </row>
+    <row r="23" ht="19" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Top 1</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>선정 근거 (컨센서스와의 차이 중심, 2줄)</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="9" t="n"/>
+      <c r="L23" s="9" t="n"/>
+      <c r="M23" s="9" t="n"/>
+      <c r="N23" s="9" t="n"/>
+      <c r="O23" s="9" t="n"/>
+      <c r="P23" s="9" t="n"/>
+      <c r="Q23" s="9" t="n"/>
     </row>
     <row r="24" ht="19" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Top 1</t>
+          <t>Top 2</t>
         </is>
       </c>
       <c r="B24" s="8" t="n"/>
-      <c r="C24" s="29" t="inlineStr">
-        <is>
-          <t>선정 근거 (컨센서스와의 차이 중심, 2줄)</t>
-        </is>
-      </c>
+      <c r="C24" s="5" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9" t="n"/>
       <c r="F24" s="9" t="n"/>
@@ -5404,7 +5376,7 @@
     <row r="25" ht="19" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Top 2</t>
+          <t>Top 3</t>
         </is>
       </c>
       <c r="B25" s="8" t="n"/>
@@ -5427,11 +5399,15 @@
     <row r="26" ht="19" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Top 3</t>
+          <t>탈락 1</t>
         </is>
       </c>
       <c r="B26" s="8" t="n"/>
-      <c r="C26" s="5" t="n"/>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>탈락 사유 (해당 지표와 수치를 명시)</t>
+        </is>
+      </c>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n"/>
       <c r="F26" s="9" t="n"/>
@@ -5450,15 +5426,11 @@
     <row r="27" ht="19" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>탈락 1</t>
+          <t>탈락 2</t>
         </is>
       </c>
       <c r="B27" s="8" t="n"/>
-      <c r="C27" s="29" t="inlineStr">
-        <is>
-          <t>탈락 사유 (해당 지표와 수치를 명시)</t>
-        </is>
-      </c>
+      <c r="C27" s="5" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="9" t="n"/>
       <c r="F27" s="9" t="n"/>
@@ -5477,7 +5449,7 @@
     <row r="28" ht="19" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>탈락 2</t>
+          <t>탈락 3</t>
         </is>
       </c>
       <c r="B28" s="8" t="n"/>
@@ -5500,7 +5472,7 @@
     <row r="29" ht="19" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>탈락 3</t>
+          <t>탈락 4</t>
         </is>
       </c>
       <c r="B29" s="8" t="n"/>
@@ -5521,50 +5493,27 @@
       <c r="Q29" s="9" t="n"/>
     </row>
     <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>탈락 4</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="n"/>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9" t="n"/>
-      <c r="G30" s="9" t="n"/>
-      <c r="H30" s="9" t="n"/>
-      <c r="I30" s="9" t="n"/>
-      <c r="J30" s="9" t="n"/>
-      <c r="K30" s="9" t="n"/>
-      <c r="L30" s="9" t="n"/>
-      <c r="M30" s="9" t="n"/>
-      <c r="N30" s="9" t="n"/>
-      <c r="O30" s="9" t="n"/>
-      <c r="P30" s="9" t="n"/>
-      <c r="Q30" s="9" t="n"/>
-    </row>
-    <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="30" t="inlineStr">
+      <c r="A30" s="30" t="inlineStr">
         <is>
           <t>탈락 5</t>
         </is>
       </c>
-      <c r="B31" s="31" t="n"/>
-      <c r="C31" s="27" t="n"/>
-      <c r="D31" s="32" t="n"/>
-      <c r="E31" s="32" t="n"/>
-      <c r="F31" s="32" t="n"/>
-      <c r="G31" s="32" t="n"/>
-      <c r="H31" s="32" t="n"/>
-      <c r="I31" s="32" t="n"/>
-      <c r="J31" s="32" t="n"/>
-      <c r="K31" s="32" t="n"/>
-      <c r="L31" s="32" t="n"/>
-      <c r="M31" s="32" t="n"/>
-      <c r="N31" s="32" t="n"/>
-      <c r="O31" s="32" t="n"/>
-      <c r="P31" s="32" t="n"/>
-      <c r="Q31" s="32" t="n"/>
+      <c r="B30" s="31" t="n"/>
+      <c r="C30" s="27" t="n"/>
+      <c r="D30" s="32" t="n"/>
+      <c r="E30" s="32" t="n"/>
+      <c r="F30" s="32" t="n"/>
+      <c r="G30" s="32" t="n"/>
+      <c r="H30" s="32" t="n"/>
+      <c r="I30" s="32" t="n"/>
+      <c r="J30" s="32" t="n"/>
+      <c r="K30" s="32" t="n"/>
+      <c r="L30" s="32" t="n"/>
+      <c r="M30" s="32" t="n"/>
+      <c r="N30" s="32" t="n"/>
+      <c r="O30" s="32" t="n"/>
+      <c r="P30" s="32" t="n"/>
+      <c r="Q30" s="32" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -5581,12 +5530,12 @@
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="K5:L5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="C31:Q31"/>
+    <mergeCell ref="C23:Q23"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="Q11:Q21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q11:Q20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Top1,Top2,Top3,보류,탈락"</formula1>
     </dataValidation>
   </dataValidations>
@@ -13277,7 +13226,7 @@
         <v>0.01410904011690083</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.07573448057211087</v>
+        <v>0.07568541860711278</v>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
@@ -13316,7 +13265,7 @@
         <v>0.008928172595490967</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.02513476766671145</v>
+        <v>0.02511848497642053</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -13355,7 +13304,7 @@
         <v>0.006652944671781102</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.08140940759045705</v>
+        <v>0.08135666932017981</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -13394,7 +13343,7 @@
         <v>0.002879689069598642</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.04220082091824706</v>
+        <v>0.04217348257535303</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -13433,7 +13382,7 @@
         <v>0.001362926842813564</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.0120927535736395</v>
+        <v>0.01208491970129921</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -13472,7 +13421,7 @@
         <v>0.0006493508750221516</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.000695436510975514</v>
+        <v>0.0006949859964740328</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -13511,7 +13460,7 @@
         <v>0.0005009476125933685</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.009410060801330396</v>
+        <v>0.009403964818758426</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -13550,7 +13499,7 @@
         <v>0.0004421512617806439</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.01046250181200551</v>
+        <v>0.01045572404190904</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -13589,7 +13538,7 @@
         <v>0.0004284782070582673</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.01002914374878634</v>
+        <v>0.01002264671472938</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -13628,7 +13577,7 @@
         <v>0.0003818562522456024</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.001461035755996035</v>
+        <v>0.00146008927449144</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -13667,7 +13616,7 @@
         <v>0.0002854257683487664</v>
       </c>
       <c r="G20" s="26" t="n">
-        <v>0.01153557892092915</v>
+        <v>0.01152810599492535</v>
       </c>
       <c r="H20" s="22" t="inlineStr">
         <is>
@@ -14176,7 +14125,7 @@
         <v>0.0160581038015037</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.0754249390983829</v>
+        <v>0.07537607765912731</v>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
@@ -14215,7 +14164,7 @@
         <v>0.008276284590010952</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.1128794574194677</v>
+        <v>0.1128063323653697</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -14254,7 +14203,7 @@
         <v>0.003161324819785457</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.03906413398447026</v>
+        <v>0.03903882763576689</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -14293,7 +14242,7 @@
         <v>0.002151577313831402</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.01741686692176065</v>
+        <v>0.01740558400664937</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -14332,7 +14281,7 @@
         <v>0.001965390089997233</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.02208062512592878</v>
+        <v>0.02206632095629718</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -14371,7 +14320,7 @@
         <v>0.0008761635412318318</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.02366960469106571</v>
+        <v>0.02365427115595595</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -14410,7 +14359,7 @@
         <v>0.0004786430947311328</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.007428995369471366</v>
+        <v>0.007424182751651389</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -14449,7 +14398,7 @@
         <v>0.0003942578315398244</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.008275075397661161</v>
+        <v>0.008269714676145019</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -14488,7 +14437,7 @@
         <v>0.0002572430235661724</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.008512390527519273</v>
+        <v>0.008506876069600551</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -14527,7 +14476,7 @@
         <v>0.0002553423818415401</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.01787086108322834</v>
+        <v>0.01785928406369473</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -14566,7 +14515,7 @@
         <v>0.0001549656677986683</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>0.002517603986320852</v>
+        <v>0.002515973043615193</v>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
@@ -14605,7 +14554,7 @@
         <v>0.0001314398050368245</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>0.006097967032441079</v>
+        <v>0.006094016675313849</v>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
@@ -14644,7 +14593,7 @@
         <v>8.433475715318468e-05</v>
       </c>
       <c r="G22" s="26" t="n">
-        <v>0.004230400140948972</v>
+        <v>0.004227659622468152</v>
       </c>
       <c r="H22" s="22" t="inlineStr">
         <is>
@@ -15153,7 +15102,7 @@
         <v>0.01846973858318185</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.2717774139331608</v>
+        <v>0.2716013523312467</v>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
@@ -15192,7 +15141,7 @@
         <v>0.006177638918416693</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.04168491846203377</v>
+        <v>0.04165791432871058</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -15231,7 +15180,7 @@
         <v>0.002248467984715008</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.1044186571375697</v>
+        <v>0.1043510131204334</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -15270,7 +15219,7 @@
         <v>0.0008082843647675407</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.001776768059198568</v>
+        <v>0.001775617041436624</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -15309,7 +15258,7 @@
         <v>0.000425932252125341</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.007346450976477239</v>
+        <v>0.007341691832188597</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -15348,7 +15297,7 @@
         <v>0.000421360986288176</v>
       </c>
       <c r="G15" s="26" t="n">
-        <v>0.009172745671472284</v>
+        <v>0.009166803425302896</v>
       </c>
       <c r="H15" s="22" t="inlineStr">
         <is>
@@ -15613,7 +15562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15703,7 +15652,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>2.96%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="C5" s="9" t="n"/>
@@ -15714,7 +15663,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>830,050원</t>
+          <t>833,191원</t>
         </is>
       </c>
       <c r="F5" s="9" t="n"/>
@@ -15725,7 +15674,7 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I5" s="9" t="n"/>
@@ -15744,7 +15693,7 @@
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>순수지주를 재료 기준으로 묶었다. 하위 테마·주요 제품(자체 사업)·보유 자회사는 기입 완료 항목이다. 지주의 재료는 자체 사업과 보유 자회사 두 갈래이며, 자체 사업이 있는 지주는 그쪽이 주가를 먼저 움직인다. SK스퀘어는 SK하이닉스 룩스루 배수가 1.8배이므로 편입 시 펀드 전체의 SK하이닉스 노출을 함께 계산한다.</t>
+          <t>순수지주를 재료 기준으로 묶었다. 하위 테마·주요 제품(자체 사업)·보유 자회사는 기입 완료 항목이다. 지주의 재료는 자체 사업과 보유 자회사 두 갈래이며, 자체 사업이 있는 지주는 그쪽이 주가를 먼저 움직인다. SK스퀘어는 SK하이닉스 룩스루 배수가 1.8배이므로 편입 시 펀드 전체의 SK하이닉스 노출을 함께 계산한다. 한화머시너리앤서비스홀딩스는 2026-08-01 (주)한화 인적분할로 신설된 지주이며, 한화비전 → 한화세미텍(HBM TC본더)으로 2단 룩스루가 걸린다 — 같은 팀의 한화비전과 합산 노출을 확인한다.</t>
         </is>
       </c>
     </row>
@@ -15868,7 +15817,7 @@
         <v>0.02476936235099287</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.2063609824853157</v>
+        <v>0.2062272986569831</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -15919,7 +15868,7 @@
         <v>0.003244636688850546</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.02358706029807158</v>
+        <v>0.02357178023649316</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -15970,7 +15919,7 @@
         <v>0.0006756851739113342</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.03444164797679919</v>
+        <v>0.03441933614585047</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -16021,7 +15970,7 @@
         <v>0.0004313540471547004</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.00499393577614464</v>
+        <v>0.004990700627498989</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -16072,7 +16021,7 @@
         <v>0.0003632700302160859</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.005169342611257159</v>
+        <v>0.005165993831357425</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -16098,114 +16047,142 @@
       <c r="Q15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>반도체·AI</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>솔브레인홀딩스</t>
         </is>
       </c>
-      <c r="C16" s="22" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>036830</t>
         </is>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="14" t="n">
         <v>41650</v>
       </c>
-      <c r="E16" s="24" t="n">
+      <c r="E16" s="15" t="n">
         <v>0.8539909999999999</v>
       </c>
-      <c r="F16" s="25" t="n">
+      <c r="F16" s="16" t="n">
         <v>0.0001603408996404638</v>
       </c>
-      <c r="G16" s="26" t="n">
-        <v>0.0085949349205134</v>
-      </c>
-      <c r="H16" s="22" t="inlineStr">
-        <is>
-          <t>가능</t>
-        </is>
-      </c>
-      <c r="I16" s="34" t="n"/>
-      <c r="J16" s="34" t="n"/>
-      <c r="K16" s="34" t="n"/>
-      <c r="L16" s="34" t="n"/>
-      <c r="M16" s="37" t="inlineStr">
-        <is>
-          <t>전자재료 일부</t>
-        </is>
-      </c>
-      <c r="N16" s="37" t="inlineStr">
-        <is>
-          <t>솔브레인 — 반도체 공정 소재</t>
-        </is>
-      </c>
-      <c r="O16" s="34" t="n"/>
-      <c r="P16" s="34" t="n"/>
-      <c r="Q16" s="34" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="G16" s="17" t="n">
+        <v>0.008589366989063344</v>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>가능</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="n"/>
+      <c r="J16" s="19" t="n"/>
+      <c r="K16" s="19" t="n"/>
+      <c r="L16" s="19" t="n"/>
+      <c r="M16" s="36" t="inlineStr">
+        <is>
+          <t>—  2020년 인적분할로 투자사업부문만 남은 순수지주</t>
+        </is>
+      </c>
+      <c r="N16" s="36" t="inlineStr">
+        <is>
+          <t>솔브레인 44.9% — 반도체·디스플레이 공정소재 · 2차전지 전해액 / 바이오헬스케어(연결 매출 11%)</t>
+        </is>
+      </c>
+      <c r="O16" s="19" t="n"/>
+      <c r="P16" s="19" t="n"/>
+      <c r="Q16" s="19" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>반도체·AI</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>한화머시너리앤서비스홀딩스</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>0220W0</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="n">
+        <v>7070</v>
+      </c>
+      <c r="E17" s="24" t="n">
+        <v>0.597525</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>0.0001121881800366376</v>
+      </c>
+      <c r="G17" s="26" t="n">
+        <v>0.00145802700150487</v>
+      </c>
+      <c r="H17" s="22" t="inlineStr">
+        <is>
+          <t>가능</t>
+        </is>
+      </c>
+      <c r="I17" s="27" t="n"/>
+      <c r="J17" s="27" t="n"/>
+      <c r="K17" s="27" t="n"/>
+      <c r="L17" s="27" t="n"/>
+      <c r="M17" s="37" t="inlineStr">
+        <is>
+          <t>—  2026-08-01 (주)한화 인적분할 신설 · 8-25 재상장</t>
+        </is>
+      </c>
+      <c r="N17" s="37" t="inlineStr">
+        <is>
+          <t>한화비전(→한화세미텍 — HBM TC본더) · 한화모멘텀 · 한화로보틱스 / 한화갤러리아 · 한화호텔앤드리조트 · 아워홈</t>
+        </is>
+      </c>
+      <c r="O17" s="27" t="n"/>
+      <c r="P17" s="27" t="n"/>
+      <c r="Q17" s="27" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>선정 결과</t>
         </is>
       </c>
-      <c r="B18" s="28" t="n"/>
-      <c r="C18" s="28" t="n"/>
-      <c r="D18" s="28" t="n"/>
-      <c r="E18" s="28" t="n"/>
-      <c r="F18" s="28" t="n"/>
-      <c r="G18" s="28" t="n"/>
-      <c r="H18" s="28" t="n"/>
-      <c r="I18" s="28" t="n"/>
-      <c r="J18" s="28" t="n"/>
-      <c r="K18" s="28" t="n"/>
-      <c r="L18" s="28" t="n"/>
-      <c r="M18" s="28" t="n"/>
-      <c r="N18" s="28" t="n"/>
-      <c r="O18" s="28" t="n"/>
-      <c r="P18" s="28" t="n"/>
-      <c r="Q18" s="28" t="n"/>
-    </row>
-    <row r="19" ht="19" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Top 1</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="29" t="inlineStr">
-        <is>
-          <t>선정 근거 (컨센서스와의 차이 중심, 2줄)</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="9" t="n"/>
-      <c r="H19" s="9" t="n"/>
-      <c r="I19" s="9" t="n"/>
-      <c r="J19" s="9" t="n"/>
-      <c r="K19" s="9" t="n"/>
-      <c r="L19" s="9" t="n"/>
-      <c r="M19" s="9" t="n"/>
-      <c r="N19" s="9" t="n"/>
-      <c r="O19" s="9" t="n"/>
-      <c r="P19" s="9" t="n"/>
-      <c r="Q19" s="9" t="n"/>
+      <c r="B19" s="28" t="n"/>
+      <c r="C19" s="28" t="n"/>
+      <c r="D19" s="28" t="n"/>
+      <c r="E19" s="28" t="n"/>
+      <c r="F19" s="28" t="n"/>
+      <c r="G19" s="28" t="n"/>
+      <c r="H19" s="28" t="n"/>
+      <c r="I19" s="28" t="n"/>
+      <c r="J19" s="28" t="n"/>
+      <c r="K19" s="28" t="n"/>
+      <c r="L19" s="28" t="n"/>
+      <c r="M19" s="28" t="n"/>
+      <c r="N19" s="28" t="n"/>
+      <c r="O19" s="28" t="n"/>
+      <c r="P19" s="28" t="n"/>
+      <c r="Q19" s="28" t="n"/>
     </row>
     <row r="20" ht="19" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Top 2</t>
+          <t>Top 1</t>
         </is>
       </c>
       <c r="B20" s="8" t="n"/>
-      <c r="C20" s="5" t="n"/>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>선정 근거 (컨센서스와의 차이 중심, 2줄)</t>
+        </is>
+      </c>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="9" t="n"/>
       <c r="F20" s="9" t="n"/>
@@ -16224,7 +16201,7 @@
     <row r="21" ht="19" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Top 3</t>
+          <t>Top 2</t>
         </is>
       </c>
       <c r="B21" s="8" t="n"/>
@@ -16247,15 +16224,11 @@
     <row r="22" ht="19" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>탈락 1</t>
+          <t>Top 3</t>
         </is>
       </c>
       <c r="B22" s="8" t="n"/>
-      <c r="C22" s="29" t="inlineStr">
-        <is>
-          <t>탈락 사유 (해당 지표와 수치를 명시)</t>
-        </is>
-      </c>
+      <c r="C22" s="5" t="n"/>
       <c r="D22" s="9" t="n"/>
       <c r="E22" s="9" t="n"/>
       <c r="F22" s="9" t="n"/>
@@ -16274,11 +16247,15 @@
     <row r="23" ht="19" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>탈락 2</t>
+          <t>탈락 1</t>
         </is>
       </c>
       <c r="B23" s="8" t="n"/>
-      <c r="C23" s="5" t="n"/>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>탈락 사유 (해당 지표와 수치를 명시)</t>
+        </is>
+      </c>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
@@ -16297,7 +16274,7 @@
     <row r="24" ht="19" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>탈락 3</t>
+          <t>탈락 2</t>
         </is>
       </c>
       <c r="B24" s="8" t="n"/>
@@ -16320,7 +16297,7 @@
     <row r="25" ht="19" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>탈락 4</t>
+          <t>탈락 3</t>
         </is>
       </c>
       <c r="B25" s="8" t="n"/>
@@ -16341,27 +16318,50 @@
       <c r="Q25" s="9" t="n"/>
     </row>
     <row r="26" ht="19" customHeight="1">
-      <c r="A26" s="30" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>탈락 4</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
+      <c r="M26" s="9" t="n"/>
+      <c r="N26" s="9" t="n"/>
+      <c r="O26" s="9" t="n"/>
+      <c r="P26" s="9" t="n"/>
+      <c r="Q26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="19" customHeight="1">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>탈락 5</t>
         </is>
       </c>
-      <c r="B26" s="31" t="n"/>
-      <c r="C26" s="27" t="n"/>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="32" t="n"/>
-      <c r="G26" s="32" t="n"/>
-      <c r="H26" s="32" t="n"/>
-      <c r="I26" s="32" t="n"/>
-      <c r="J26" s="32" t="n"/>
-      <c r="K26" s="32" t="n"/>
-      <c r="L26" s="32" t="n"/>
-      <c r="M26" s="32" t="n"/>
-      <c r="N26" s="32" t="n"/>
-      <c r="O26" s="32" t="n"/>
-      <c r="P26" s="32" t="n"/>
-      <c r="Q26" s="32" t="n"/>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="27" t="n"/>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="32" t="n"/>
+      <c r="F27" s="32" t="n"/>
+      <c r="G27" s="32" t="n"/>
+      <c r="H27" s="32" t="n"/>
+      <c r="I27" s="32" t="n"/>
+      <c r="J27" s="32" t="n"/>
+      <c r="K27" s="32" t="n"/>
+      <c r="L27" s="32" t="n"/>
+      <c r="M27" s="32" t="n"/>
+      <c r="N27" s="32" t="n"/>
+      <c r="O27" s="32" t="n"/>
+      <c r="P27" s="32" t="n"/>
+      <c r="Q27" s="32" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -16372,18 +16372,18 @@
     <mergeCell ref="C24:Q24"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A7:Q7"/>
-    <mergeCell ref="C19:Q19"/>
+    <mergeCell ref="C27:Q27"/>
+    <mergeCell ref="C26:Q26"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="K5:L5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="C26:Q26"/>
     <mergeCell ref="C23:Q23"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="C22:Q22"/>
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="Q11:Q16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q11:Q17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Top1,Top2,Top3,보류,탈락"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16648,7 +16648,7 @@
         <v>0.003981709229656787</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.04591531860298274</v>
+        <v>0.04588557395117873</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -16687,7 +16687,7 @@
         <v>0.001682575803002602</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.03978639742316887</v>
+        <v>0.03976062318106633</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -16726,7 +16726,7 @@
         <v>0.00144169467048583</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.02158535876796402</v>
+        <v>0.02157137543952043</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -16765,7 +16765,7 @@
         <v>0.001032778822602822</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.09214017867969347</v>
+        <v>0.09208048885034292</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -16804,7 +16804,7 @@
         <v>0.0009989859647379395</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.02236953050140822</v>
+        <v>0.02235503917441696</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -16843,7 +16843,7 @@
         <v>0.0009532282452170343</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.02408232665603634</v>
+        <v>0.02406672575326992</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -16882,7 +16882,7 @@
         <v>0.0009200776964838283</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.0132690111738058</v>
+        <v>0.01326041530364401</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -16921,7 +16921,7 @@
         <v>0.0008972082244628038</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.01995510700633003</v>
+        <v>0.01994217978013026</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -16960,7 +16960,7 @@
         <v>0.0008947953876749694</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.02589830330190712</v>
+        <v>0.02588152598145137</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -16999,7 +16999,7 @@
         <v>0.0008019701712281371</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>0.01071013499098789</v>
+        <v>0.01070319680029742</v>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
@@ -17038,7 +17038,7 @@
         <v>0.0007227406545307931</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>0.03747515441933334</v>
+        <v>0.03745087743610812</v>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
@@ -17077,7 +17077,7 @@
         <v>0.0006433909747687682</v>
       </c>
       <c r="G22" s="17" t="n">
-        <v>0.02441250422801285</v>
+        <v>0.02439668943112109</v>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
@@ -17116,7 +17116,7 @@
         <v>0.0005546047393335222</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>0.0265999306423572</v>
+        <v>0.02658269879688512</v>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
@@ -17155,7 +17155,7 @@
         <v>0.0005446875314015777</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>0.05355067495493943</v>
+        <v>0.0535159840014871</v>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
@@ -17194,7 +17194,7 @@
         <v>0.0004746504891523217</v>
       </c>
       <c r="G25" s="17" t="n">
-        <v>0.06706731930772761</v>
+        <v>0.06702387206351949</v>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
@@ -17233,7 +17233,7 @@
         <v>0.0004714507720456159</v>
       </c>
       <c r="G26" s="17" t="n">
-        <v>0.02676501942834545</v>
+        <v>0.0267476806358107</v>
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
@@ -17272,7 +17272,7 @@
         <v>0.0004449163265518243</v>
       </c>
       <c r="G27" s="17" t="n">
-        <v>0.01419763559498972</v>
+        <v>0.01418843814760043</v>
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
@@ -17311,7 +17311,7 @@
         <v>0.0004188375619298773</v>
       </c>
       <c r="G28" s="17" t="n">
-        <v>0.006923410962382342</v>
+        <v>0.006918925869941781</v>
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
@@ -17350,7 +17350,7 @@
         <v>0.0004114062273985186</v>
       </c>
       <c r="G29" s="17" t="n">
-        <v>0.04189127944451909</v>
+        <v>0.04186414162736756</v>
       </c>
       <c r="H29" s="13" t="inlineStr">
         <is>
@@ -17389,7 +17389,7 @@
         <v>0.0003799244432260686</v>
       </c>
       <c r="G30" s="17" t="n">
-        <v>0.008192531004667034</v>
+        <v>0.008187223756682226</v>
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
@@ -17428,7 +17428,7 @@
         <v>0.0003521558855070466</v>
       </c>
       <c r="G31" s="17" t="n">
-        <v>0.005674927018346182</v>
+        <v>0.005671250713067033</v>
       </c>
       <c r="H31" s="13" t="inlineStr">
         <is>
@@ -17467,7 +17467,7 @@
         <v>0.0003346030658337858</v>
       </c>
       <c r="G32" s="17" t="n">
-        <v>0.05251887004251285</v>
+        <v>0.05248484750820218</v>
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
@@ -17506,7 +17506,7 @@
         <v>0.0003068037163294393</v>
       </c>
       <c r="G33" s="17" t="n">
-        <v>0.009100519327602422</v>
+        <v>0.009094623870772952</v>
       </c>
       <c r="H33" s="13" t="inlineStr">
         <is>
@@ -17545,7 +17545,7 @@
         <v>0.000269981434951078</v>
       </c>
       <c r="G34" s="17" t="n">
-        <v>0.01535325709690749</v>
+        <v>0.01534331102007954</v>
       </c>
       <c r="H34" s="13" t="inlineStr">
         <is>
@@ -17584,7 +17584,7 @@
         <v>0.000265552674998433</v>
       </c>
       <c r="G35" s="17" t="n">
-        <v>0.001774704449373715</v>
+        <v>0.001773554768450054</v>
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
@@ -17623,7 +17623,7 @@
         <v>0.0002545740892467367</v>
       </c>
       <c r="G36" s="17" t="n">
-        <v>0.009162427622348018</v>
+        <v>0.009156492060370048</v>
       </c>
       <c r="H36" s="13" t="inlineStr">
         <is>
@@ -17662,7 +17662,7 @@
         <v>0.0002502540393166702</v>
       </c>
       <c r="G37" s="17" t="n">
-        <v>0.005355067495493943</v>
+        <v>0.00535159840014871</v>
       </c>
       <c r="H37" s="13" t="inlineStr">
         <is>
@@ -17701,7 +17701,7 @@
         <v>0.0002462400296919628</v>
       </c>
       <c r="G38" s="17" t="n">
-        <v>0.01018391448565033</v>
+        <v>0.01017731718872211</v>
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
@@ -17740,7 +17740,7 @@
         <v>0.0002317678905894583</v>
       </c>
       <c r="G39" s="17" t="n">
-        <v>0.003468928115578157</v>
+        <v>0.003466680890423885</v>
       </c>
       <c r="H39" s="13" t="inlineStr">
         <is>
@@ -17779,7 +17779,7 @@
         <v>0.0002228912196957348</v>
       </c>
       <c r="G40" s="17" t="n">
-        <v>0.01021486863302313</v>
+        <v>0.01020825128352066</v>
       </c>
       <c r="H40" s="13" t="inlineStr">
         <is>
@@ -17818,7 +17818,7 @@
         <v>0.0001949510540999654</v>
       </c>
       <c r="G41" s="17" t="n">
-        <v>0.01083395158047907</v>
+        <v>0.01082693317949161</v>
       </c>
       <c r="H41" s="13" t="inlineStr">
         <is>
@@ -17857,7 +17857,7 @@
         <v>0.0001935802563886604</v>
       </c>
       <c r="G42" s="17" t="n">
-        <v>0.004127219649706314</v>
+        <v>0.004124545973139661</v>
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
@@ -17896,7 +17896,7 @@
         <v>0.0001799235363328888</v>
       </c>
       <c r="G43" s="17" t="n">
-        <v>0.002410296275428487</v>
+        <v>0.002408734848313562</v>
       </c>
       <c r="H43" s="13" t="inlineStr">
         <is>
@@ -17935,7 +17935,7 @@
         <v>0.000160999543438746</v>
       </c>
       <c r="G44" s="17" t="n">
-        <v>0.00643846265354185</v>
+        <v>0.006434291718097871</v>
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
@@ -17974,7 +17974,7 @@
         <v>0.0001586266984208755</v>
       </c>
       <c r="G45" s="17" t="n">
-        <v>0.008171894906418502</v>
+        <v>0.008166601026816529</v>
       </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
@@ -18013,7 +18013,7 @@
         <v>0.0001433618586010542</v>
       </c>
       <c r="G46" s="17" t="n">
-        <v>0.006345600211423458</v>
+        <v>0.006341489433702228</v>
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
@@ -18052,7 +18052,7 @@
         <v>0.0001364432823972635</v>
       </c>
       <c r="G47" s="17" t="n">
-        <v>0.006397190457044787</v>
+        <v>0.006393046258366474</v>
       </c>
       <c r="H47" s="13" t="inlineStr">
         <is>
@@ -18091,7 +18091,7 @@
         <v>0.0001342724615318878</v>
       </c>
       <c r="G48" s="26" t="n">
-        <v>0.002245207489440235</v>
+        <v>0.002243753009387975</v>
       </c>
       <c r="H48" s="22" t="inlineStr">
         <is>
@@ -18601,7 +18601,7 @@
         <v>0.005882627892602164</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.04251036239197504</v>
+        <v>0.04248282352333851</v>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
@@ -18640,7 +18640,7 @@
         <v>0.003203435590293298</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.04550259663801211</v>
+        <v>0.04547311935386476</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -18679,7 +18679,7 @@
         <v>0.002869549747751826</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.007119453895743392</v>
+        <v>0.007114841803665915</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -18718,7 +18718,7 @@
         <v>0.00190512399469963</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.07635356351956682</v>
+        <v>0.07630410050308373</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -18757,7 +18757,7 @@
         <v>0.001808067724092511</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.04343898681315896</v>
+        <v>0.04341084636729493</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -18796,7 +18796,7 @@
         <v>0.001291546790561711</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.01465162975645742</v>
+        <v>0.0146421382046458</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -18835,7 +18835,7 @@
         <v>0.001162202704474837</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.009441014948703193</v>
+        <v>0.009434898913556974</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -18874,7 +18874,7 @@
         <v>0.0008251785406425193</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.0420976404270044</v>
+        <v>0.04207036892602454</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -18913,7 +18913,7 @@
         <v>0.0006180046498070448</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.004467715270807085</v>
+        <v>0.004464821015923683</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -18952,7 +18952,7 @@
         <v>0.0005488108143132292</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.007253588534358847</v>
+        <v>0.007248889547792954</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -18991,7 +18991,7 @@
         <v>0.0004285474885752474</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>0.00272602857863102</v>
+        <v>0.002724262615258746</v>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
@@ -19030,7 +19030,7 @@
         <v>0.000421233125277164</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>0.007367087074725771</v>
+        <v>0.007362314562054295</v>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
@@ -19069,7 +19069,7 @@
         <v>0.0001980142734753852</v>
       </c>
       <c r="G22" s="17" t="n">
-        <v>0.002038846506954919</v>
+        <v>0.002037525710730992</v>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
@@ -19108,7 +19108,7 @@
         <v>0.0001339600375637175</v>
       </c>
       <c r="G23" s="26" t="n">
-        <v>0.004756620646286527</v>
+        <v>0.004753539234043459</v>
       </c>
       <c r="H23" s="22" t="inlineStr">
         <is>
@@ -19617,7 +19617,7 @@
         <v>0.01036713806237023</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.01823936365635324</v>
+        <v>0.01825149491863809</v>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
@@ -19656,7 +19656,7 @@
         <v>0.005483378600008368</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.04119726338621783</v>
+        <v>0.04122466427678464</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -19695,7 +19695,7 @@
         <v>0.00473761564105866</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.1481154821281586</v>
+        <v>0.14821399585901</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -19734,7 +19734,7 @@
         <v>0.00470770911956226</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.5689750449180264</v>
+        <v>0.569353478378397</v>
       </c>
       <c r="H13" s="38" t="inlineStr">
         <is>
@@ -19773,7 +19773,7 @@
         <v>0.003778672891096895</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.006633457663882532</v>
+        <v>0.006637869671685662</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -19812,7 +19812,7 @@
         <v>0.001078751521356633</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.03967378985575677</v>
+        <v>0.03970017746223482</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -19851,7 +19851,7 @@
         <v>0.00103190707711952</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.03042715190004172</v>
+        <v>0.03044738943503663</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -19890,7 +19890,7 @@
         <v>0.001026679420541536</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.005903459930536607</v>
+        <v>0.005907386406380542</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -19929,7 +19929,7 @@
         <v>0.0006395585240246021</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.007807801843612932</v>
+        <v>0.007812994924567813</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -19968,7 +19968,7 @@
         <v>0.0006345128018367362</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.01091822696830426</v>
+        <v>0.01092548883760702</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -20007,7 +20007,7 @@
         <v>0.0006123962265178528</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>0.01447299853938007</v>
+        <v>0.01448262473822326</v>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
@@ -20046,7 +20046,7 @@
         <v>0.0004196477238425305</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>0.01121445793256058</v>
+        <v>0.01122191682932504</v>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
@@ -20085,7 +20085,7 @@
         <v>0.0004021707571038495</v>
       </c>
       <c r="G22" s="17" t="n">
-        <v>0.01007185278471479</v>
+        <v>0.01007855171841268</v>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
@@ -20124,7 +20124,7 @@
         <v>0.0003788089920272105</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>0.01379589919250849</v>
+        <v>0.01380507504286779</v>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
@@ -20163,7 +20163,7 @@
         <v>0.0003191724385356625</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>0.01055851794027873</v>
+        <v>0.01056554056194943</v>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
@@ -20202,7 +20202,7 @@
         <v>0.0002866358479610606</v>
       </c>
       <c r="G25" s="17" t="n">
-        <v>0.01054793826298387</v>
+        <v>0.0105549538479595</v>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
@@ -20241,7 +20241,7 @@
         <v>0.0002594921381783792</v>
       </c>
       <c r="G26" s="17" t="n">
-        <v>0.02611064356373539</v>
+        <v>0.02612801012714548</v>
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
@@ -20280,7 +20280,7 @@
         <v>0.0002262865772921241</v>
       </c>
       <c r="G27" s="26" t="n">
-        <v>0.005649547675459764</v>
+        <v>0.005653305270622239</v>
       </c>
       <c r="H27" s="22" t="inlineStr">
         <is>
@@ -20789,7 +20789,7 @@
         <v>0.008937112164238861</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0.09595767306445704</v>
+        <v>0.09602149588865863</v>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
@@ -20828,7 +20828,7 @@
         <v>0.004740520019882954</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>0.01743530818194324</v>
+        <v>0.01744690465540346</v>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
@@ -20867,7 +20867,7 @@
         <v>0.004504629034136633</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.07173021205920824</v>
+        <v>0.07177792085172056</v>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
@@ -20906,7 +20906,7 @@
         <v>0.003420141228479796</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>0.004379986400075547</v>
+        <v>0.004382899591830724</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -20945,7 +20945,7 @@
         <v>0.001952905710841255</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>0.04908970264818971</v>
+        <v>0.04912235291327189</v>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
@@ -20984,7 +20984,7 @@
         <v>0.0007489112312443477</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>0.01011417149389426</v>
+        <v>0.0101208985743724</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
@@ -21023,7 +21023,7 @@
         <v>0.0003289617854565952</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.009733303111278993</v>
+        <v>0.009739776870734943</v>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
@@ -21062,7 +21062,7 @@
         <v>0.0003182727175888644</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>0.006866210564369638</v>
+        <v>0.006870777379464107</v>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
@@ -21101,7 +21101,7 @@
         <v>0.0003168538546516871</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>0.01052677890839413</v>
+        <v>0.01053378041997964</v>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
@@ -21140,7 +21140,7 @@
         <v>0.0002571827542790434</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>0.003209874091263094</v>
+        <v>0.003212009024544545</v>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
@@ -21179,7 +21179,7 @@
         <v>0.0002052080981992106</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>0.004475203495729363</v>
+        <v>0.004478180017740088</v>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
@@ -21218,7 +21218,7 @@
         <v>0.0001425263497919449</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>0.002570861582653038</v>
+        <v>0.002572571499552817</v>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
@@ -21257,7 +21257,7 @@
         <v>0.0001079116892175179</v>
       </c>
       <c r="G22" s="26" t="n">
-        <v>0.002139210749022405</v>
+        <v>0.002140633568763702</v>
       </c>
       <c r="H22" s="22" t="inlineStr">
         <is>

</xml_diff>